<commit_message>
Docs: Implementacion de script de entregables y actualizacion de documentacion Carpeta N3
</commit_message>
<xml_diff>
--- a/Carpeta_N3_Base_de_datos_y_codigo/diccionario_variables.xlsx
+++ b/Carpeta_N3_Base_de_datos_y_codigo/diccionario_variables.xlsx
@@ -413,326 +413,294 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>Variable Dataset</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>definicion</t>
+          <t>Nombre Formal</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>unidad_medida</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>frecuencia</t>
+          <t>Unidad de Medida</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>fuente_exacta</t>
+          <t>Fuente</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>url_o_endpoint</t>
+          <t>Descripción</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>fecha</t>
+          <t>banco</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Fecha de corte del reporte mensual (fin de mes)</t>
+          <t>Entidad Bancaria</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fecha (AAAA-MM-DD)</t>
+          <t>Cualitativa / Identificador</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SBS - Reporte B-2402</t>
+          <t>SBS Perú</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://intranet2.sbs.gob.pe/estadistica/financiera/{anio}/{mes}/B-2402-{abrev}{anio}.XLS</t>
+          <t>Nombre estandarizado de la institución de banca múltiple.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>fecha</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nombre de la empresa bancaria supervisada por la SBS</t>
+          <t>Periodo Mensual</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Temporal / Identificador</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>YYYY-MM-DD</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SBS - Reporte B-2402</t>
+          <t>SBS Perú</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://intranet2.sbs.gob.pe/estadistica/financiera/{anio}/{mes}/B-2402-{abrev}{anio}.XLS</t>
+          <t>Fecha correspondiente al último día del mes evaluado (2018-01 a 2025-12).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>apr_total</t>
+          <t>ratio_capital_global_pct</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Activos y Contingentes Ponderados por Riesgo Total (suma de riesgo de crédito, mercado y operacional)</t>
+          <t>Ratio de Capital Global</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Miles de soles</t>
+          <t>Endógena (Y)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Porcentaje (%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SBS - Reporte B-2402</t>
+          <t>SBS Reporte B-2402</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://intranet2.sbs.gob.pe/estadistica/financiera/{anio}/{mes}/B-2402-{abrev}{anio}.XLS</t>
+          <t>Patrimonio Efectivo / APR. Métrica regulatoria principal de solvencia bancaria.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ratio_capital_global_pct</t>
+          <t>roe_pct</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ratio de Capital Global: Patrimonio Efectivo Total / Activos Ponderados por Riesgo Total</t>
+          <t>Rentabilidad del Patrimonio (ROE)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Porcentaje</t>
+          <t>Exógena (X1)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Porcentaje (%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SBS - Reporte B-2402</t>
+          <t>SBS Reporte B-2201</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://intranet2.sbs.gob.pe/estadistica/financiera/{anio}/{mes}/B-2402-{abrev}{anio}.XLS</t>
+          <t>(Utilidad Neta Anualizada / Patrimonio) * 100. Métrica de rentabilidad bancaria.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>patrimonio_efectivo_nivel1_apr_pct</t>
+          <t>cartera_atrasada_pct</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Patrimonio Efectivo de Nivel 1 sobre Activos Ponderados por Riesgo (disponible solo en el formato de reporte 2021-2025)</t>
+          <t>Ratio de Cartera Atrasada</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Porcentaje</t>
+          <t>Exógena (X2)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Porcentaje (%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SBS - Reporte B-2402</t>
+          <t>SBS Reporte B-2362</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://intranet2.sbs.gob.pe/estadistica/financiera/{anio}/{mes}/B-2402-{abrev}{anio}.XLS</t>
+          <t>Total Créditos Atrasados / Total Créditos Directos. Métrica de riesgo de crédito.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>capital_ordinario_nivel1_apr_pct</t>
+          <t>apr_total_soles</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Capital Ordinario de Nivel 1 sobre Activos Ponderados por Riesgo (disponible solo en el formato de reporte 2021-2025)</t>
+          <t>Activos Ponderados por Riesgo (APR)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Porcentaje</t>
+          <t>Exógena / Control (X3)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Miles de S/.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SBS - Reporte B-2402</t>
+          <t>SBS Reporte B-2402</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://intranet2.sbs.gob.pe/estadistica/financiera/{anio}/{mes}/B-2402-{abrev}{anio}.XLS</t>
+          <t>Suma total de activos y contingentes ponderados por riesgo del banco.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>patrimonio_efectivo_estimado</t>
+          <t>ln_apr_total_soles</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Patrimonio Efectivo Total estimado, calculado como (ratio_capital_global_pct / 100) x apr_total</t>
+          <t>Logaritmo del Tamaño del Banco</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Miles de soles</t>
+          <t>Exógena / Control (X3)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Logaritmo natural</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Calculado a partir de SBS - Reporte B-2402</t>
+          <t>Transformación propia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>N/A - variable derivada</t>
+          <t>ln(apr_total_soles). Escala operativa del banco para controlar heterogeneidad.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>fuente_dato</t>
+          <t>banco</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Indica si la observación proviene directamente de un reporte real de la SBS ('SBS_original') o fue completada mediante interpolacion lineal por ausencia de reporte ese mes ('interpolado'), segun autorizacion del docente</t>
+          <t>Entidad Bancaria de Banca Múltiple</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Categorica (SBS_original / interpolado)</t>
+          <t>Cualitativa / Identificador</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Generado en 03_limpieza_datos.py</t>
+          <t>SBS Perú (Reportes B-2402, B-2201, B-2362)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>N/A - variable derivada</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ratio_capital_global (Banco Mundial GFDD.SI.05)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Bank regulatory capital to risk-weighted assets - agregado nacional Peru</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Porcentaje</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Anual</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>World Bank Open Data - GFDD</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>https://api.worldbank.org/v2/country/PER/indicator/GFDD.SI.05</t>
+          <t>Nombre estandarizado de las 16 instituciones de banca múltiple evaluadas en el Perú (BCP, BBVA, Interbank, Scotiabank, BanBif, Pichincha, Mibanco, GNB, Falabella, Ripley, Bancom, Alfin, Citibank, ICBC, Santander, Bank of China).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correccion de scraping, limpieza, analisis y documentacion
</commit_message>
<xml_diff>
--- a/Carpeta_N3_Base_de_datos_y_codigo/diccionario_variables.xlsx
+++ b/Carpeta_N3_Base_de_datos_y_codigo/diccionario_variables.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Entidad Bancaria</t>
+          <t>Entidad Bancaria de Banca Múltiple</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SBS Perú</t>
+          <t>SBS Perú (Reportes B-2402, B-2201, B-2362)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Nombre estandarizado de la institución de banca múltiple.</t>
+          <t>Nombre estandarizado de las 16 entidades del panel: Alfin Banco, BANCOM, Banco BBVA Perú, Banco Falabella Perú, Banco GNB, Banco ICBC, Banco Interamericano de Finanzas, Banco Pichincha, Banco Ripley, Banco Santander Perú, Banco de Crédito del Perú, Bank of China, Citibank, Interbank, Mibanco, Scotiabank Perú.</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Fecha correspondiente al último día del mes evaluado (2018-01 a 2025-12).</t>
+          <t>Último día del mes evaluado (2018-01 a 2025-12).</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>(Utilidad Neta Anualizada / Patrimonio) * 100. Métrica de rentabilidad bancaria.</t>
+          <t>(Resultado neto acumulado / meses transcurridos × 12) / Patrimonio × 100.</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Total Créditos Atrasados / Total Créditos Directos. Métrica de riesgo de crédito.</t>
+          <t>Créditos atrasados / Créditos directos totales (fila 'Total Créditos Directos').</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Suma total de activos y contingentes ponderados por riesgo del banco.</t>
+          <t>Activos y contingentes ponderados por riesgo total (2018-2020: requerimiento total × 10).</t>
         </is>
       </c>
     </row>
@@ -663,44 +663,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Transformación propia</t>
+          <t>Transformación propia (04_analisis.py)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ln(apr_total_soles). Escala operativa del banco para controlar heterogeneidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>banco</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Entidad Bancaria de Banca Múltiple</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Cualitativa / Identificador</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Texto</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>SBS Perú (Reportes B-2402, B-2201, B-2362)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Nombre estandarizado de las 16 instituciones de banca múltiple evaluadas en el Perú (BCP, BBVA, Interbank, Scotiabank, BanBif, Pichincha, Mibanco, GNB, Falabella, Ripley, Bancom, Alfin, Citibank, ICBC, Santander, Bank of China).</t>
+          <t>ln(apr_total_soles). Escala del banco para controlar heterogeneidad.</t>
         </is>
       </c>
     </row>

</xml_diff>